<commit_message>
Lista para el proveedor: se suma Valentino Born in Roma Green Stravaganza Donna 100 ml
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UyW4b53zwrRCyiu74Lz3oD
</commit_message>
<xml_diff>
--- a/novaparfum/data/proveedor/NovaParfum-lista-100ml.xlsx
+++ b/novaparfum/data/proveedor/NovaParfum-lista-100ml.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Resumen" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Lista 100 ml'!$A$5:$J$301</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Lista 100 ml'!$A$5:$J$302</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sin versión de 100 ml'!$A$5:$J$112</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J301"/>
+  <dimension ref="A1:J302"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -8010,7 +8010,7 @@
       </c>
       <c r="E223" s="6" t="inlineStr">
         <is>
-          <t>Donna Born in Roma Intense</t>
+          <t>Donna Born in Roma Green Stravaganza</t>
         </is>
       </c>
       <c r="F223" s="6" t="inlineStr">
@@ -8046,10 +8046,14 @@
       </c>
       <c r="E224" s="11" t="inlineStr">
         <is>
-          <t>Donna Born in Roma Purple Melancholia</t>
-        </is>
-      </c>
-      <c r="F224" s="11" t="inlineStr"/>
+          <t>Donna Born in Roma Intense</t>
+        </is>
+      </c>
+      <c r="F224" s="11" t="inlineStr">
+        <is>
+          <t>EDP</t>
+        </is>
+      </c>
       <c r="G224" s="10" t="n">
         <v>100</v>
       </c>
@@ -8078,7 +8082,7 @@
       </c>
       <c r="E225" s="6" t="inlineStr">
         <is>
-          <t>Donna Born in Roma Yellow Dream</t>
+          <t>Donna Born in Roma Purple Melancholia</t>
         </is>
       </c>
       <c r="F225" s="6" t="inlineStr"/>
@@ -8100,7 +8104,7 @@
       </c>
       <c r="C226" s="11" t="inlineStr">
         <is>
-          <t>Caballero</t>
+          <t>Dama</t>
         </is>
       </c>
       <c r="D226" s="11" t="inlineStr">
@@ -8110,7 +8114,7 @@
       </c>
       <c r="E226" s="11" t="inlineStr">
         <is>
-          <t>Uomo Born in Roma</t>
+          <t>Donna Born in Roma Yellow Dream</t>
         </is>
       </c>
       <c r="F226" s="11" t="inlineStr"/>
@@ -8142,7 +8146,7 @@
       </c>
       <c r="E227" s="6" t="inlineStr">
         <is>
-          <t>Uomo Born in Roma Coral Fantasy</t>
+          <t>Uomo Born in Roma</t>
         </is>
       </c>
       <c r="F227" s="6" t="inlineStr"/>
@@ -8174,7 +8178,7 @@
       </c>
       <c r="E228" s="11" t="inlineStr">
         <is>
-          <t>Uomo Born in Roma Extradose</t>
+          <t>Uomo Born in Roma Coral Fantasy</t>
         </is>
       </c>
       <c r="F228" s="11" t="inlineStr"/>
@@ -8206,7 +8210,7 @@
       </c>
       <c r="E229" s="6" t="inlineStr">
         <is>
-          <t>Uomo Born in Roma Green Stravaganza</t>
+          <t>Uomo Born in Roma Extradose</t>
         </is>
       </c>
       <c r="F229" s="6" t="inlineStr"/>
@@ -8238,7 +8242,7 @@
       </c>
       <c r="E230" s="11" t="inlineStr">
         <is>
-          <t>Uomo Born in Roma Purple Melancholia</t>
+          <t>Uomo Born in Roma Green Stravaganza</t>
         </is>
       </c>
       <c r="F230" s="11" t="inlineStr"/>
@@ -8260,7 +8264,7 @@
       </c>
       <c r="C231" s="6" t="inlineStr">
         <is>
-          <t>Dama</t>
+          <t>Caballero</t>
         </is>
       </c>
       <c r="D231" s="6" t="inlineStr">
@@ -8270,7 +8274,7 @@
       </c>
       <c r="E231" s="6" t="inlineStr">
         <is>
-          <t>Voce Viva</t>
+          <t>Uomo Born in Roma Purple Melancholia</t>
         </is>
       </c>
       <c r="F231" s="6" t="inlineStr"/>
@@ -8297,12 +8301,12 @@
       </c>
       <c r="D232" s="11" t="inlineStr">
         <is>
-          <t>Versace</t>
+          <t>Valentino</t>
         </is>
       </c>
       <c r="E232" s="11" t="inlineStr">
         <is>
-          <t>Dylan Blue pour Femme</t>
+          <t>Voce Viva</t>
         </is>
       </c>
       <c r="F232" s="11" t="inlineStr"/>
@@ -8324,7 +8328,7 @@
       </c>
       <c r="C233" s="6" t="inlineStr">
         <is>
-          <t>Caballero</t>
+          <t>Dama</t>
         </is>
       </c>
       <c r="D233" s="6" t="inlineStr">
@@ -8334,7 +8338,7 @@
       </c>
       <c r="E233" s="6" t="inlineStr">
         <is>
-          <t>Dylan Blue pour Homme</t>
+          <t>Dylan Blue pour Femme</t>
         </is>
       </c>
       <c r="F233" s="6" t="inlineStr"/>
@@ -8356,7 +8360,7 @@
       </c>
       <c r="C234" s="11" t="inlineStr">
         <is>
-          <t>Dama</t>
+          <t>Caballero</t>
         </is>
       </c>
       <c r="D234" s="11" t="inlineStr">
@@ -8366,14 +8370,10 @@
       </c>
       <c r="E234" s="11" t="inlineStr">
         <is>
-          <t>Dylan Purple</t>
-        </is>
-      </c>
-      <c r="F234" s="11" t="inlineStr">
-        <is>
-          <t>EDP</t>
-        </is>
-      </c>
+          <t>Dylan Blue pour Homme</t>
+        </is>
+      </c>
+      <c r="F234" s="11" t="inlineStr"/>
       <c r="G234" s="10" t="n">
         <v>100</v>
       </c>
@@ -8402,12 +8402,12 @@
       </c>
       <c r="E235" s="6" t="inlineStr">
         <is>
-          <t>Dylan Turquoise</t>
+          <t>Dylan Purple</t>
         </is>
       </c>
       <c r="F235" s="6" t="inlineStr">
         <is>
-          <t>EDT</t>
+          <t>EDP</t>
         </is>
       </c>
       <c r="G235" s="5" t="n">
@@ -8428,7 +8428,7 @@
       </c>
       <c r="C236" s="11" t="inlineStr">
         <is>
-          <t>Caballero</t>
+          <t>Dama</t>
         </is>
       </c>
       <c r="D236" s="11" t="inlineStr">
@@ -8438,10 +8438,14 @@
       </c>
       <c r="E236" s="11" t="inlineStr">
         <is>
-          <t>Eros</t>
-        </is>
-      </c>
-      <c r="F236" s="11" t="inlineStr"/>
+          <t>Dylan Turquoise</t>
+        </is>
+      </c>
+      <c r="F236" s="11" t="inlineStr">
+        <is>
+          <t>EDT</t>
+        </is>
+      </c>
       <c r="G236" s="10" t="n">
         <v>100</v>
       </c>
@@ -8470,14 +8474,10 @@
       </c>
       <c r="E237" s="6" t="inlineStr">
         <is>
-          <t>Eros EDP</t>
-        </is>
-      </c>
-      <c r="F237" s="6" t="inlineStr">
-        <is>
-          <t>EDP</t>
-        </is>
-      </c>
+          <t>Eros</t>
+        </is>
+      </c>
+      <c r="F237" s="6" t="inlineStr"/>
       <c r="G237" s="5" t="n">
         <v>100</v>
       </c>
@@ -8506,7 +8506,7 @@
       </c>
       <c r="E238" s="11" t="inlineStr">
         <is>
-          <t>Eros Energy</t>
+          <t>Eros EDP</t>
         </is>
       </c>
       <c r="F238" s="11" t="inlineStr">
@@ -8542,10 +8542,14 @@
       </c>
       <c r="E239" s="6" t="inlineStr">
         <is>
-          <t>Eros Flame</t>
-        </is>
-      </c>
-      <c r="F239" s="6" t="inlineStr"/>
+          <t>Eros Energy</t>
+        </is>
+      </c>
+      <c r="F239" s="6" t="inlineStr">
+        <is>
+          <t>EDP</t>
+        </is>
+      </c>
       <c r="G239" s="5" t="n">
         <v>100</v>
       </c>
@@ -8574,14 +8578,10 @@
       </c>
       <c r="E240" s="11" t="inlineStr">
         <is>
-          <t>Eros Najim</t>
-        </is>
-      </c>
-      <c r="F240" s="11" t="inlineStr">
-        <is>
-          <t>Parfum</t>
-        </is>
-      </c>
+          <t>Eros Flame</t>
+        </is>
+      </c>
+      <c r="F240" s="11" t="inlineStr"/>
       <c r="G240" s="10" t="n">
         <v>100</v>
       </c>
@@ -8610,10 +8610,14 @@
       </c>
       <c r="E241" s="6" t="inlineStr">
         <is>
-          <t>Pour Homme</t>
-        </is>
-      </c>
-      <c r="F241" s="6" t="inlineStr"/>
+          <t>Eros Najim</t>
+        </is>
+      </c>
+      <c r="F241" s="6" t="inlineStr">
+        <is>
+          <t>Parfum</t>
+        </is>
+      </c>
       <c r="G241" s="5" t="n">
         <v>100</v>
       </c>
@@ -8632,7 +8636,7 @@
       </c>
       <c r="C242" s="11" t="inlineStr">
         <is>
-          <t>Dama</t>
+          <t>Caballero</t>
         </is>
       </c>
       <c r="D242" s="11" t="inlineStr">
@@ -8642,7 +8646,7 @@
       </c>
       <c r="E242" s="11" t="inlineStr">
         <is>
-          <t>Versense</t>
+          <t>Pour Homme</t>
         </is>
       </c>
       <c r="F242" s="11" t="inlineStr"/>
@@ -8669,19 +8673,15 @@
       </c>
       <c r="D243" s="6" t="inlineStr">
         <is>
-          <t>Victoria's Secret</t>
+          <t>Versace</t>
         </is>
       </c>
       <c r="E243" s="6" t="inlineStr">
         <is>
-          <t>Bombshell</t>
-        </is>
-      </c>
-      <c r="F243" s="6" t="inlineStr">
-        <is>
-          <t>EDP</t>
-        </is>
-      </c>
+          <t>Versense</t>
+        </is>
+      </c>
+      <c r="F243" s="6" t="inlineStr"/>
       <c r="G243" s="5" t="n">
         <v>100</v>
       </c>
@@ -8705,15 +8705,19 @@
       </c>
       <c r="D244" s="11" t="inlineStr">
         <is>
-          <t>Viktor&amp;Rolf</t>
+          <t>Victoria's Secret</t>
         </is>
       </c>
       <c r="E244" s="11" t="inlineStr">
         <is>
-          <t>Flowerbomb</t>
-        </is>
-      </c>
-      <c r="F244" s="11" t="inlineStr"/>
+          <t>Bombshell</t>
+        </is>
+      </c>
+      <c r="F244" s="11" t="inlineStr">
+        <is>
+          <t>EDP</t>
+        </is>
+      </c>
       <c r="G244" s="10" t="n">
         <v>100</v>
       </c>
@@ -8732,17 +8736,17 @@
       </c>
       <c r="C245" s="6" t="inlineStr">
         <is>
-          <t>Caballero</t>
+          <t>Dama</t>
         </is>
       </c>
       <c r="D245" s="6" t="inlineStr">
         <is>
-          <t>Yves Saint Laurent</t>
+          <t>Viktor&amp;Rolf</t>
         </is>
       </c>
       <c r="E245" s="6" t="inlineStr">
         <is>
-          <t>La Nuit de L'Homme</t>
+          <t>Flowerbomb</t>
         </is>
       </c>
       <c r="F245" s="6" t="inlineStr"/>
@@ -8774,14 +8778,10 @@
       </c>
       <c r="E246" s="11" t="inlineStr">
         <is>
-          <t>MYSLF EDP</t>
-        </is>
-      </c>
-      <c r="F246" s="11" t="inlineStr">
-        <is>
-          <t>EDP</t>
-        </is>
-      </c>
+          <t>La Nuit de L'Homme</t>
+        </is>
+      </c>
+      <c r="F246" s="11" t="inlineStr"/>
       <c r="G246" s="10" t="n">
         <v>100</v>
       </c>
@@ -8810,10 +8810,14 @@
       </c>
       <c r="E247" s="6" t="inlineStr">
         <is>
-          <t>MYSLF L'Absolu</t>
-        </is>
-      </c>
-      <c r="F247" s="6" t="inlineStr"/>
+          <t>MYSLF EDP</t>
+        </is>
+      </c>
+      <c r="F247" s="6" t="inlineStr">
+        <is>
+          <t>EDP</t>
+        </is>
+      </c>
       <c r="G247" s="5" t="n">
         <v>100</v>
       </c>
@@ -8842,14 +8846,10 @@
       </c>
       <c r="E248" s="11" t="inlineStr">
         <is>
-          <t>Y EDP</t>
-        </is>
-      </c>
-      <c r="F248" s="11" t="inlineStr">
-        <is>
-          <t>EDP</t>
-        </is>
-      </c>
+          <t>MYSLF L'Absolu</t>
+        </is>
+      </c>
+      <c r="F248" s="11" t="inlineStr"/>
       <c r="G248" s="10" t="n">
         <v>100</v>
       </c>
@@ -8878,12 +8878,12 @@
       </c>
       <c r="E249" s="6" t="inlineStr">
         <is>
-          <t>Y Le Parfum</t>
+          <t>Y EDP</t>
         </is>
       </c>
       <c r="F249" s="6" t="inlineStr">
         <is>
-          <t>Parfum</t>
+          <t>EDP</t>
         </is>
       </c>
       <c r="G249" s="5" t="n">
@@ -8899,25 +8899,29 @@
       </c>
       <c r="B250" s="11" t="inlineStr">
         <is>
-          <t>Nicho</t>
+          <t>Diseñador</t>
         </is>
       </c>
       <c r="C250" s="11" t="inlineStr">
         <is>
-          <t>Unisex</t>
+          <t>Caballero</t>
         </is>
       </c>
       <c r="D250" s="11" t="inlineStr">
         <is>
-          <t>Amouage</t>
+          <t>Yves Saint Laurent</t>
         </is>
       </c>
       <c r="E250" s="11" t="inlineStr">
         <is>
-          <t>Guidance</t>
-        </is>
-      </c>
-      <c r="F250" s="11" t="inlineStr"/>
+          <t>Y Le Parfum</t>
+        </is>
+      </c>
+      <c r="F250" s="11" t="inlineStr">
+        <is>
+          <t>Parfum</t>
+        </is>
+      </c>
       <c r="G250" s="10" t="n">
         <v>100</v>
       </c>
@@ -8936,7 +8940,7 @@
       </c>
       <c r="C251" s="6" t="inlineStr">
         <is>
-          <t>Caballero</t>
+          <t>Unisex</t>
         </is>
       </c>
       <c r="D251" s="6" t="inlineStr">
@@ -8946,7 +8950,7 @@
       </c>
       <c r="E251" s="6" t="inlineStr">
         <is>
-          <t>Interlude Man</t>
+          <t>Guidance</t>
         </is>
       </c>
       <c r="F251" s="6" t="inlineStr"/>
@@ -8978,7 +8982,7 @@
       </c>
       <c r="E252" s="11" t="inlineStr">
         <is>
-          <t>Reflection Man</t>
+          <t>Interlude Man</t>
         </is>
       </c>
       <c r="F252" s="11" t="inlineStr"/>
@@ -9000,17 +9004,17 @@
       </c>
       <c r="C253" s="6" t="inlineStr">
         <is>
-          <t>Unisex</t>
+          <t>Caballero</t>
         </is>
       </c>
       <c r="D253" s="6" t="inlineStr">
         <is>
-          <t>Byredo</t>
+          <t>Amouage</t>
         </is>
       </c>
       <c r="E253" s="6" t="inlineStr">
         <is>
-          <t>Bal d'Afrique</t>
+          <t>Reflection Man</t>
         </is>
       </c>
       <c r="F253" s="6" t="inlineStr"/>
@@ -9032,7 +9036,7 @@
       </c>
       <c r="C254" s="11" t="inlineStr">
         <is>
-          <t>Dama</t>
+          <t>Unisex</t>
         </is>
       </c>
       <c r="D254" s="11" t="inlineStr">
@@ -9042,14 +9046,10 @@
       </c>
       <c r="E254" s="11" t="inlineStr">
         <is>
-          <t>Blanche</t>
-        </is>
-      </c>
-      <c r="F254" s="11" t="inlineStr">
-        <is>
-          <t>EDP</t>
-        </is>
-      </c>
+          <t>Bal d'Afrique</t>
+        </is>
+      </c>
+      <c r="F254" s="11" t="inlineStr"/>
       <c r="G254" s="10" t="n">
         <v>100</v>
       </c>
@@ -9068,7 +9068,7 @@
       </c>
       <c r="C255" s="6" t="inlineStr">
         <is>
-          <t>Unisex</t>
+          <t>Dama</t>
         </is>
       </c>
       <c r="D255" s="6" t="inlineStr">
@@ -9078,10 +9078,14 @@
       </c>
       <c r="E255" s="6" t="inlineStr">
         <is>
-          <t>Gypsy Water</t>
-        </is>
-      </c>
-      <c r="F255" s="6" t="inlineStr"/>
+          <t>Blanche</t>
+        </is>
+      </c>
+      <c r="F255" s="6" t="inlineStr">
+        <is>
+          <t>EDP</t>
+        </is>
+      </c>
       <c r="G255" s="5" t="n">
         <v>100</v>
       </c>
@@ -9110,7 +9114,7 @@
       </c>
       <c r="E256" s="11" t="inlineStr">
         <is>
-          <t>Mojave Ghost</t>
+          <t>Gypsy Water</t>
         </is>
       </c>
       <c r="F256" s="11" t="inlineStr"/>
@@ -9132,24 +9136,20 @@
       </c>
       <c r="C257" s="6" t="inlineStr">
         <is>
-          <t>Caballero</t>
+          <t>Unisex</t>
         </is>
       </c>
       <c r="D257" s="6" t="inlineStr">
         <is>
-          <t>Creed</t>
+          <t>Byredo</t>
         </is>
       </c>
       <c r="E257" s="6" t="inlineStr">
         <is>
-          <t>Absolu Aventus</t>
-        </is>
-      </c>
-      <c r="F257" s="6" t="inlineStr">
-        <is>
-          <t>EDP</t>
-        </is>
-      </c>
+          <t>Mojave Ghost</t>
+        </is>
+      </c>
+      <c r="F257" s="6" t="inlineStr"/>
       <c r="G257" s="5" t="n">
         <v>100</v>
       </c>
@@ -9178,10 +9178,14 @@
       </c>
       <c r="E258" s="11" t="inlineStr">
         <is>
-          <t>Aventus</t>
-        </is>
-      </c>
-      <c r="F258" s="11" t="inlineStr"/>
+          <t>Absolu Aventus</t>
+        </is>
+      </c>
+      <c r="F258" s="11" t="inlineStr">
+        <is>
+          <t>EDP</t>
+        </is>
+      </c>
       <c r="G258" s="10" t="n">
         <v>100</v>
       </c>
@@ -9200,7 +9204,7 @@
       </c>
       <c r="C259" s="6" t="inlineStr">
         <is>
-          <t>Dama</t>
+          <t>Caballero</t>
         </is>
       </c>
       <c r="D259" s="6" t="inlineStr">
@@ -9210,7 +9214,7 @@
       </c>
       <c r="E259" s="6" t="inlineStr">
         <is>
-          <t>Aventus for Her</t>
+          <t>Aventus</t>
         </is>
       </c>
       <c r="F259" s="6" t="inlineStr"/>
@@ -9232,7 +9236,7 @@
       </c>
       <c r="C260" s="11" t="inlineStr">
         <is>
-          <t>Caballero</t>
+          <t>Dama</t>
         </is>
       </c>
       <c r="D260" s="11" t="inlineStr">
@@ -9242,7 +9246,7 @@
       </c>
       <c r="E260" s="11" t="inlineStr">
         <is>
-          <t>Green Irish Tweed</t>
+          <t>Aventus for Her</t>
         </is>
       </c>
       <c r="F260" s="11" t="inlineStr"/>
@@ -9264,7 +9268,7 @@
       </c>
       <c r="C261" s="6" t="inlineStr">
         <is>
-          <t>Unisex</t>
+          <t>Caballero</t>
         </is>
       </c>
       <c r="D261" s="6" t="inlineStr">
@@ -9274,14 +9278,10 @@
       </c>
       <c r="E261" s="6" t="inlineStr">
         <is>
-          <t>Millésime Impérial</t>
-        </is>
-      </c>
-      <c r="F261" s="6" t="inlineStr">
-        <is>
-          <t>EDP</t>
-        </is>
-      </c>
+          <t>Green Irish Tweed</t>
+        </is>
+      </c>
+      <c r="F261" s="6" t="inlineStr"/>
       <c r="G261" s="5" t="n">
         <v>100</v>
       </c>
@@ -9310,10 +9310,14 @@
       </c>
       <c r="E262" s="11" t="inlineStr">
         <is>
-          <t>Royal Oud</t>
-        </is>
-      </c>
-      <c r="F262" s="11" t="inlineStr"/>
+          <t>Millésime Impérial</t>
+        </is>
+      </c>
+      <c r="F262" s="11" t="inlineStr">
+        <is>
+          <t>EDP</t>
+        </is>
+      </c>
       <c r="G262" s="10" t="n">
         <v>100</v>
       </c>
@@ -9342,7 +9346,7 @@
       </c>
       <c r="E263" s="6" t="inlineStr">
         <is>
-          <t>Silver Mountain Water</t>
+          <t>Royal Oud</t>
         </is>
       </c>
       <c r="F263" s="6" t="inlineStr"/>
@@ -9364,7 +9368,7 @@
       </c>
       <c r="C264" s="11" t="inlineStr">
         <is>
-          <t>Caballero</t>
+          <t>Unisex</t>
         </is>
       </c>
       <c r="D264" s="11" t="inlineStr">
@@ -9374,7 +9378,7 @@
       </c>
       <c r="E264" s="11" t="inlineStr">
         <is>
-          <t>Viking</t>
+          <t>Silver Mountain Water</t>
         </is>
       </c>
       <c r="F264" s="11" t="inlineStr"/>
@@ -9396,24 +9400,20 @@
       </c>
       <c r="C265" s="6" t="inlineStr">
         <is>
-          <t>Unisex</t>
+          <t>Caballero</t>
         </is>
       </c>
       <c r="D265" s="6" t="inlineStr">
         <is>
-          <t>Escentric Molecules</t>
+          <t>Creed</t>
         </is>
       </c>
       <c r="E265" s="6" t="inlineStr">
         <is>
-          <t>Molecule 01</t>
-        </is>
-      </c>
-      <c r="F265" s="6" t="inlineStr">
-        <is>
-          <t>EDT</t>
-        </is>
-      </c>
+          <t>Viking</t>
+        </is>
+      </c>
+      <c r="F265" s="6" t="inlineStr"/>
       <c r="G265" s="5" t="n">
         <v>100</v>
       </c>
@@ -9432,22 +9432,22 @@
       </c>
       <c r="C266" s="11" t="inlineStr">
         <is>
-          <t>Dama</t>
+          <t>Unisex</t>
         </is>
       </c>
       <c r="D266" s="11" t="inlineStr">
         <is>
-          <t>Jo Malone</t>
+          <t>Escentric Molecules</t>
         </is>
       </c>
       <c r="E266" s="11" t="inlineStr">
         <is>
-          <t>English Pear &amp; Freesia</t>
+          <t>Molecule 01</t>
         </is>
       </c>
       <c r="F266" s="11" t="inlineStr">
         <is>
-          <t>Cologne</t>
+          <t>EDT</t>
         </is>
       </c>
       <c r="G266" s="10" t="n">
@@ -9468,7 +9468,7 @@
       </c>
       <c r="C267" s="6" t="inlineStr">
         <is>
-          <t>Unisex</t>
+          <t>Dama</t>
         </is>
       </c>
       <c r="D267" s="6" t="inlineStr">
@@ -9478,7 +9478,7 @@
       </c>
       <c r="E267" s="6" t="inlineStr">
         <is>
-          <t>Wood Sage &amp; Sea Salt</t>
+          <t>English Pear &amp; Freesia</t>
         </is>
       </c>
       <c r="F267" s="6" t="inlineStr">
@@ -9504,22 +9504,22 @@
       </c>
       <c r="C268" s="11" t="inlineStr">
         <is>
-          <t>Dama</t>
+          <t>Unisex</t>
         </is>
       </c>
       <c r="D268" s="11" t="inlineStr">
         <is>
-          <t>Kayali</t>
+          <t>Jo Malone</t>
         </is>
       </c>
       <c r="E268" s="11" t="inlineStr">
         <is>
-          <t>Vanilla 28</t>
+          <t>Wood Sage &amp; Sea Salt</t>
         </is>
       </c>
       <c r="F268" s="11" t="inlineStr">
         <is>
-          <t>EDP</t>
+          <t>Cologne</t>
         </is>
       </c>
       <c r="G268" s="10" t="n">
@@ -9550,7 +9550,7 @@
       </c>
       <c r="E269" s="6" t="inlineStr">
         <is>
-          <t>Yum Pistachio Gelato 33</t>
+          <t>Vanilla 28</t>
         </is>
       </c>
       <c r="F269" s="6" t="inlineStr">
@@ -9576,20 +9576,24 @@
       </c>
       <c r="C270" s="11" t="inlineStr">
         <is>
-          <t>Unisex</t>
+          <t>Dama</t>
         </is>
       </c>
       <c r="D270" s="11" t="inlineStr">
         <is>
-          <t>Le Labo</t>
+          <t>Kayali</t>
         </is>
       </c>
       <c r="E270" s="11" t="inlineStr">
         <is>
-          <t>Another 13</t>
-        </is>
-      </c>
-      <c r="F270" s="11" t="inlineStr"/>
+          <t>Yum Pistachio Gelato 33</t>
+        </is>
+      </c>
+      <c r="F270" s="11" t="inlineStr">
+        <is>
+          <t>EDP</t>
+        </is>
+      </c>
       <c r="G270" s="10" t="n">
         <v>100</v>
       </c>
@@ -9618,14 +9622,10 @@
       </c>
       <c r="E271" s="6" t="inlineStr">
         <is>
-          <t>Rose 31</t>
-        </is>
-      </c>
-      <c r="F271" s="6" t="inlineStr">
-        <is>
-          <t>EDP</t>
-        </is>
-      </c>
+          <t>Another 13</t>
+        </is>
+      </c>
+      <c r="F271" s="6" t="inlineStr"/>
       <c r="G271" s="5" t="n">
         <v>100</v>
       </c>
@@ -9654,10 +9654,14 @@
       </c>
       <c r="E272" s="11" t="inlineStr">
         <is>
-          <t>Santal 33</t>
-        </is>
-      </c>
-      <c r="F272" s="11" t="inlineStr"/>
+          <t>Rose 31</t>
+        </is>
+      </c>
+      <c r="F272" s="11" t="inlineStr">
+        <is>
+          <t>EDP</t>
+        </is>
+      </c>
       <c r="G272" s="10" t="n">
         <v>100</v>
       </c>
@@ -9676,17 +9680,17 @@
       </c>
       <c r="C273" s="6" t="inlineStr">
         <is>
-          <t>Caballero</t>
+          <t>Unisex</t>
         </is>
       </c>
       <c r="D273" s="6" t="inlineStr">
         <is>
-          <t>Louis Vuitton</t>
+          <t>Le Labo</t>
         </is>
       </c>
       <c r="E273" s="6" t="inlineStr">
         <is>
-          <t>Imagination</t>
+          <t>Santal 33</t>
         </is>
       </c>
       <c r="F273" s="6" t="inlineStr"/>
@@ -9718,14 +9722,10 @@
       </c>
       <c r="E274" s="11" t="inlineStr">
         <is>
-          <t>L'Immensité</t>
-        </is>
-      </c>
-      <c r="F274" s="11" t="inlineStr">
-        <is>
-          <t>EDP</t>
-        </is>
-      </c>
+          <t>Imagination</t>
+        </is>
+      </c>
+      <c r="F274" s="11" t="inlineStr"/>
       <c r="G274" s="10" t="n">
         <v>100</v>
       </c>
@@ -9744,7 +9744,7 @@
       </c>
       <c r="C275" s="6" t="inlineStr">
         <is>
-          <t>Unisex</t>
+          <t>Caballero</t>
         </is>
       </c>
       <c r="D275" s="6" t="inlineStr">
@@ -9754,10 +9754,14 @@
       </c>
       <c r="E275" s="6" t="inlineStr">
         <is>
-          <t>Ombre Nomade</t>
-        </is>
-      </c>
-      <c r="F275" s="6" t="inlineStr"/>
+          <t>L'Immensité</t>
+        </is>
+      </c>
+      <c r="F275" s="6" t="inlineStr">
+        <is>
+          <t>EDP</t>
+        </is>
+      </c>
       <c r="G275" s="5" t="n">
         <v>100</v>
       </c>
@@ -9781,12 +9785,12 @@
       </c>
       <c r="D276" s="11" t="inlineStr">
         <is>
-          <t>Maison Margiela</t>
+          <t>Louis Vuitton</t>
         </is>
       </c>
       <c r="E276" s="11" t="inlineStr">
         <is>
-          <t>Replica By the Fireplace</t>
+          <t>Ombre Nomade</t>
         </is>
       </c>
       <c r="F276" s="11" t="inlineStr"/>
@@ -9808,7 +9812,7 @@
       </c>
       <c r="C277" s="6" t="inlineStr">
         <is>
-          <t>Caballero</t>
+          <t>Unisex</t>
         </is>
       </c>
       <c r="D277" s="6" t="inlineStr">
@@ -9818,7 +9822,7 @@
       </c>
       <c r="E277" s="6" t="inlineStr">
         <is>
-          <t>Replica Jazz Club</t>
+          <t>Replica By the Fireplace</t>
         </is>
       </c>
       <c r="F277" s="6" t="inlineStr"/>
@@ -9840,7 +9844,7 @@
       </c>
       <c r="C278" s="11" t="inlineStr">
         <is>
-          <t>Unisex</t>
+          <t>Caballero</t>
         </is>
       </c>
       <c r="D278" s="11" t="inlineStr">
@@ -9850,14 +9854,10 @@
       </c>
       <c r="E278" s="11" t="inlineStr">
         <is>
-          <t>Replica Lazy Sunday Morning</t>
-        </is>
-      </c>
-      <c r="F278" s="11" t="inlineStr">
-        <is>
-          <t>EDT</t>
-        </is>
-      </c>
+          <t>Replica Jazz Club</t>
+        </is>
+      </c>
+      <c r="F278" s="11" t="inlineStr"/>
       <c r="G278" s="10" t="n">
         <v>100</v>
       </c>
@@ -9881,15 +9881,19 @@
       </c>
       <c r="D279" s="6" t="inlineStr">
         <is>
-          <t>Montale</t>
+          <t>Maison Margiela</t>
         </is>
       </c>
       <c r="E279" s="6" t="inlineStr">
         <is>
-          <t>Arabians Tonka</t>
-        </is>
-      </c>
-      <c r="F279" s="6" t="inlineStr"/>
+          <t>Replica Lazy Sunday Morning</t>
+        </is>
+      </c>
+      <c r="F279" s="6" t="inlineStr">
+        <is>
+          <t>EDT</t>
+        </is>
+      </c>
       <c r="G279" s="5" t="n">
         <v>100</v>
       </c>
@@ -9908,7 +9912,7 @@
       </c>
       <c r="C280" s="11" t="inlineStr">
         <is>
-          <t>Caballero</t>
+          <t>Unisex</t>
         </is>
       </c>
       <c r="D280" s="11" t="inlineStr">
@@ -9918,7 +9922,7 @@
       </c>
       <c r="E280" s="11" t="inlineStr">
         <is>
-          <t>Black Aoud</t>
+          <t>Arabians Tonka</t>
         </is>
       </c>
       <c r="F280" s="11" t="inlineStr"/>
@@ -9940,7 +9944,7 @@
       </c>
       <c r="C281" s="6" t="inlineStr">
         <is>
-          <t>Unisex</t>
+          <t>Caballero</t>
         </is>
       </c>
       <c r="D281" s="6" t="inlineStr">
@@ -9950,7 +9954,7 @@
       </c>
       <c r="E281" s="6" t="inlineStr">
         <is>
-          <t>Intense Café</t>
+          <t>Black Aoud</t>
         </is>
       </c>
       <c r="F281" s="6" t="inlineStr"/>
@@ -9972,7 +9976,7 @@
       </c>
       <c r="C282" s="11" t="inlineStr">
         <is>
-          <t>Dama</t>
+          <t>Unisex</t>
         </is>
       </c>
       <c r="D282" s="11" t="inlineStr">
@@ -9982,14 +9986,10 @@
       </c>
       <c r="E282" s="11" t="inlineStr">
         <is>
-          <t>Roses Musk</t>
-        </is>
-      </c>
-      <c r="F282" s="11" t="inlineStr">
-        <is>
-          <t>EDP</t>
-        </is>
-      </c>
+          <t>Intense Café</t>
+        </is>
+      </c>
+      <c r="F282" s="11" t="inlineStr"/>
       <c r="G282" s="10" t="n">
         <v>100</v>
       </c>
@@ -10008,20 +10008,24 @@
       </c>
       <c r="C283" s="6" t="inlineStr">
         <is>
-          <t>Unisex</t>
+          <t>Dama</t>
         </is>
       </c>
       <c r="D283" s="6" t="inlineStr">
         <is>
-          <t>Nishane</t>
+          <t>Montale</t>
         </is>
       </c>
       <c r="E283" s="6" t="inlineStr">
         <is>
-          <t>Ani</t>
-        </is>
-      </c>
-      <c r="F283" s="6" t="inlineStr"/>
+          <t>Roses Musk</t>
+        </is>
+      </c>
+      <c r="F283" s="6" t="inlineStr">
+        <is>
+          <t>EDP</t>
+        </is>
+      </c>
       <c r="G283" s="5" t="n">
         <v>100</v>
       </c>
@@ -10050,7 +10054,7 @@
       </c>
       <c r="E284" s="11" t="inlineStr">
         <is>
-          <t>Hacivat</t>
+          <t>Ani</t>
         </is>
       </c>
       <c r="F284" s="11" t="inlineStr"/>
@@ -10082,14 +10086,10 @@
       </c>
       <c r="E285" s="6" t="inlineStr">
         <is>
-          <t>Wulong Cha</t>
-        </is>
-      </c>
-      <c r="F285" s="6" t="inlineStr">
-        <is>
-          <t>Extrait</t>
-        </is>
-      </c>
+          <t>Hacivat</t>
+        </is>
+      </c>
+      <c r="F285" s="6" t="inlineStr"/>
       <c r="G285" s="5" t="n">
         <v>100</v>
       </c>
@@ -10113,15 +10113,19 @@
       </c>
       <c r="D286" s="11" t="inlineStr">
         <is>
-          <t>Tom Ford</t>
+          <t>Nishane</t>
         </is>
       </c>
       <c r="E286" s="11" t="inlineStr">
         <is>
-          <t>Bitter Peach</t>
-        </is>
-      </c>
-      <c r="F286" s="11" t="inlineStr"/>
+          <t>Wulong Cha</t>
+        </is>
+      </c>
+      <c r="F286" s="11" t="inlineStr">
+        <is>
+          <t>Extrait</t>
+        </is>
+      </c>
       <c r="G286" s="10" t="n">
         <v>100</v>
       </c>
@@ -10150,14 +10154,10 @@
       </c>
       <c r="E287" s="6" t="inlineStr">
         <is>
-          <t>Fucking Fabulous</t>
-        </is>
-      </c>
-      <c r="F287" s="6" t="inlineStr">
-        <is>
-          <t>EDP</t>
-        </is>
-      </c>
+          <t>Bitter Peach</t>
+        </is>
+      </c>
+      <c r="F287" s="6" t="inlineStr"/>
       <c r="G287" s="5" t="n">
         <v>100</v>
       </c>
@@ -10186,10 +10186,14 @@
       </c>
       <c r="E288" s="11" t="inlineStr">
         <is>
-          <t>Lost Cherry</t>
-        </is>
-      </c>
-      <c r="F288" s="11" t="inlineStr"/>
+          <t>Fucking Fabulous</t>
+        </is>
+      </c>
+      <c r="F288" s="11" t="inlineStr">
+        <is>
+          <t>EDP</t>
+        </is>
+      </c>
       <c r="G288" s="10" t="n">
         <v>100</v>
       </c>
@@ -10218,14 +10222,10 @@
       </c>
       <c r="E289" s="6" t="inlineStr">
         <is>
-          <t>Neroli Portofino</t>
-        </is>
-      </c>
-      <c r="F289" s="6" t="inlineStr">
-        <is>
-          <t>EDP</t>
-        </is>
-      </c>
+          <t>Lost Cherry</t>
+        </is>
+      </c>
+      <c r="F289" s="6" t="inlineStr"/>
       <c r="G289" s="5" t="n">
         <v>100</v>
       </c>
@@ -10244,7 +10244,7 @@
       </c>
       <c r="C290" s="11" t="inlineStr">
         <is>
-          <t>Caballero</t>
+          <t>Unisex</t>
         </is>
       </c>
       <c r="D290" s="11" t="inlineStr">
@@ -10254,7 +10254,7 @@
       </c>
       <c r="E290" s="11" t="inlineStr">
         <is>
-          <t>Noir Extreme</t>
+          <t>Neroli Portofino</t>
         </is>
       </c>
       <c r="F290" s="11" t="inlineStr">
@@ -10280,7 +10280,7 @@
       </c>
       <c r="C291" s="6" t="inlineStr">
         <is>
-          <t>Unisex</t>
+          <t>Caballero</t>
         </is>
       </c>
       <c r="D291" s="6" t="inlineStr">
@@ -10290,10 +10290,14 @@
       </c>
       <c r="E291" s="6" t="inlineStr">
         <is>
-          <t>Oud Wood</t>
-        </is>
-      </c>
-      <c r="F291" s="6" t="inlineStr"/>
+          <t>Noir Extreme</t>
+        </is>
+      </c>
+      <c r="F291" s="6" t="inlineStr">
+        <is>
+          <t>EDP</t>
+        </is>
+      </c>
       <c r="G291" s="5" t="n">
         <v>100</v>
       </c>
@@ -10322,14 +10326,10 @@
       </c>
       <c r="E292" s="11" t="inlineStr">
         <is>
-          <t>Rose Prick</t>
-        </is>
-      </c>
-      <c r="F292" s="11" t="inlineStr">
-        <is>
-          <t>EDP</t>
-        </is>
-      </c>
+          <t>Oud Wood</t>
+        </is>
+      </c>
+      <c r="F292" s="11" t="inlineStr"/>
       <c r="G292" s="10" t="n">
         <v>100</v>
       </c>
@@ -10358,10 +10358,14 @@
       </c>
       <c r="E293" s="6" t="inlineStr">
         <is>
-          <t>Soleil Blanc</t>
-        </is>
-      </c>
-      <c r="F293" s="6" t="inlineStr"/>
+          <t>Rose Prick</t>
+        </is>
+      </c>
+      <c r="F293" s="6" t="inlineStr">
+        <is>
+          <t>EDP</t>
+        </is>
+      </c>
       <c r="G293" s="5" t="n">
         <v>100</v>
       </c>
@@ -10390,7 +10394,7 @@
       </c>
       <c r="E294" s="11" t="inlineStr">
         <is>
-          <t>Tobacco Vanille</t>
+          <t>Soleil Blanc</t>
         </is>
       </c>
       <c r="F294" s="11" t="inlineStr"/>
@@ -10422,14 +10426,10 @@
       </c>
       <c r="E295" s="6" t="inlineStr">
         <is>
-          <t>Tuscan Leather</t>
-        </is>
-      </c>
-      <c r="F295" s="6" t="inlineStr">
-        <is>
-          <t>EDP</t>
-        </is>
-      </c>
+          <t>Tobacco Vanille</t>
+        </is>
+      </c>
+      <c r="F295" s="6" t="inlineStr"/>
       <c r="G295" s="5" t="n">
         <v>100</v>
       </c>
@@ -10448,20 +10448,24 @@
       </c>
       <c r="C296" s="11" t="inlineStr">
         <is>
-          <t>Caballero</t>
+          <t>Unisex</t>
         </is>
       </c>
       <c r="D296" s="11" t="inlineStr">
         <is>
-          <t>Xerjoff</t>
+          <t>Tom Ford</t>
         </is>
       </c>
       <c r="E296" s="11" t="inlineStr">
         <is>
-          <t>40 Knots</t>
-        </is>
-      </c>
-      <c r="F296" s="11" t="inlineStr"/>
+          <t>Tuscan Leather</t>
+        </is>
+      </c>
+      <c r="F296" s="11" t="inlineStr">
+        <is>
+          <t>EDP</t>
+        </is>
+      </c>
       <c r="G296" s="10" t="n">
         <v>100</v>
       </c>
@@ -10480,7 +10484,7 @@
       </c>
       <c r="C297" s="6" t="inlineStr">
         <is>
-          <t>Unisex</t>
+          <t>Caballero</t>
         </is>
       </c>
       <c r="D297" s="6" t="inlineStr">
@@ -10490,7 +10494,7 @@
       </c>
       <c r="E297" s="6" t="inlineStr">
         <is>
-          <t>Alexandria II</t>
+          <t>40 Knots</t>
         </is>
       </c>
       <c r="F297" s="6" t="inlineStr"/>
@@ -10522,14 +10526,10 @@
       </c>
       <c r="E298" s="11" t="inlineStr">
         <is>
-          <t>Erba Gold</t>
-        </is>
-      </c>
-      <c r="F298" s="11" t="inlineStr">
-        <is>
-          <t>EDP</t>
-        </is>
-      </c>
+          <t>Alexandria II</t>
+        </is>
+      </c>
+      <c r="F298" s="11" t="inlineStr"/>
       <c r="G298" s="10" t="n">
         <v>100</v>
       </c>
@@ -10558,10 +10558,14 @@
       </c>
       <c r="E299" s="6" t="inlineStr">
         <is>
-          <t>Erba Pura</t>
-        </is>
-      </c>
-      <c r="F299" s="6" t="inlineStr"/>
+          <t>Erba Gold</t>
+        </is>
+      </c>
+      <c r="F299" s="6" t="inlineStr">
+        <is>
+          <t>EDP</t>
+        </is>
+      </c>
       <c r="G299" s="5" t="n">
         <v>100</v>
       </c>
@@ -10590,14 +10594,10 @@
       </c>
       <c r="E300" s="11" t="inlineStr">
         <is>
-          <t>More Than Words</t>
-        </is>
-      </c>
-      <c r="F300" s="11" t="inlineStr">
-        <is>
-          <t>EDP</t>
-        </is>
-      </c>
+          <t>Erba Pura</t>
+        </is>
+      </c>
+      <c r="F300" s="11" t="inlineStr"/>
       <c r="G300" s="10" t="n">
         <v>100</v>
       </c>
@@ -10626,10 +10626,14 @@
       </c>
       <c r="E301" s="6" t="inlineStr">
         <is>
-          <t>Naxos</t>
-        </is>
-      </c>
-      <c r="F301" s="6" t="inlineStr"/>
+          <t>More Than Words</t>
+        </is>
+      </c>
+      <c r="F301" s="6" t="inlineStr">
+        <is>
+          <t>EDP</t>
+        </is>
+      </c>
       <c r="G301" s="5" t="n">
         <v>100</v>
       </c>
@@ -10637,13 +10641,45 @@
       <c r="I301" s="8" t="n"/>
       <c r="J301" s="9" t="n"/>
     </row>
+    <row r="302">
+      <c r="A302" s="10" t="n">
+        <v>296</v>
+      </c>
+      <c r="B302" s="11" t="inlineStr">
+        <is>
+          <t>Nicho</t>
+        </is>
+      </c>
+      <c r="C302" s="11" t="inlineStr">
+        <is>
+          <t>Unisex</t>
+        </is>
+      </c>
+      <c r="D302" s="11" t="inlineStr">
+        <is>
+          <t>Xerjoff</t>
+        </is>
+      </c>
+      <c r="E302" s="11" t="inlineStr">
+        <is>
+          <t>Naxos</t>
+        </is>
+      </c>
+      <c r="F302" s="11" t="inlineStr"/>
+      <c r="G302" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="H302" s="7" t="n"/>
+      <c r="I302" s="8" t="n"/>
+      <c r="J302" s="9" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:J301"/>
+  <autoFilter ref="A5:J302"/>
   <dataValidations count="2">
-    <dataValidation sqref="H7:H301" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H7:H302" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="I7:I301" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Poné el precio en pesos, sin puntos ni símbolo." type="decimal" operator="greaterThan">
+    <dataValidation sqref="I7:I302" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Poné el precio en pesos, sin puntos ni símbolo." type="decimal" operator="greaterThan">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -14519,19 +14555,19 @@
         </is>
       </c>
       <c r="C4" s="14">
-        <f>COUNTIFS('Lista 100 ml'!$B$7:$B$301,B4)</f>
+        <f>COUNTIFS('Lista 100 ml'!$B$7:$B$302,B4)</f>
         <v/>
       </c>
       <c r="D4" s="14">
-        <f>COUNTIFS('Lista 100 ml'!$B$7:$B$301,B4,'Lista 100 ml'!$H$7:$H$301,"Sí")</f>
+        <f>COUNTIFS('Lista 100 ml'!$B$7:$B$302,B4,'Lista 100 ml'!$H$7:$H$302,"Sí")</f>
         <v/>
       </c>
       <c r="E4" s="14">
-        <f>COUNTIFS('Lista 100 ml'!$B$7:$B$301,B4,'Lista 100 ml'!$H$7:$H$301,"No")</f>
+        <f>COUNTIFS('Lista 100 ml'!$B$7:$B$302,B4,'Lista 100 ml'!$H$7:$H$302,"No")</f>
         <v/>
       </c>
       <c r="F4" s="14">
-        <f>COUNTIFS('Lista 100 ml'!$B$7:$B$301,B4,'Lista 100 ml'!$I$7:$I$301,"&gt;0")</f>
+        <f>COUNTIFS('Lista 100 ml'!$B$7:$B$302,B4,'Lista 100 ml'!$I$7:$I$302,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -14547,19 +14583,19 @@
         </is>
       </c>
       <c r="C5" s="14">
-        <f>COUNTIFS('Lista 100 ml'!$B$7:$B$301,B5)</f>
+        <f>COUNTIFS('Lista 100 ml'!$B$7:$B$302,B5)</f>
         <v/>
       </c>
       <c r="D5" s="14">
-        <f>COUNTIFS('Lista 100 ml'!$B$7:$B$301,B5,'Lista 100 ml'!$H$7:$H$301,"Sí")</f>
+        <f>COUNTIFS('Lista 100 ml'!$B$7:$B$302,B5,'Lista 100 ml'!$H$7:$H$302,"Sí")</f>
         <v/>
       </c>
       <c r="E5" s="14">
-        <f>COUNTIFS('Lista 100 ml'!$B$7:$B$301,B5,'Lista 100 ml'!$H$7:$H$301,"No")</f>
+        <f>COUNTIFS('Lista 100 ml'!$B$7:$B$302,B5,'Lista 100 ml'!$H$7:$H$302,"No")</f>
         <v/>
       </c>
       <c r="F5" s="14">
-        <f>COUNTIFS('Lista 100 ml'!$B$7:$B$301,B5,'Lista 100 ml'!$I$7:$I$301,"&gt;0")</f>
+        <f>COUNTIFS('Lista 100 ml'!$B$7:$B$302,B5,'Lista 100 ml'!$I$7:$I$302,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -14575,19 +14611,19 @@
         </is>
       </c>
       <c r="C6" s="14">
-        <f>COUNTIFS('Lista 100 ml'!$B$7:$B$301,B6)</f>
+        <f>COUNTIFS('Lista 100 ml'!$B$7:$B$302,B6)</f>
         <v/>
       </c>
       <c r="D6" s="14">
-        <f>COUNTIFS('Lista 100 ml'!$B$7:$B$301,B6,'Lista 100 ml'!$H$7:$H$301,"Sí")</f>
+        <f>COUNTIFS('Lista 100 ml'!$B$7:$B$302,B6,'Lista 100 ml'!$H$7:$H$302,"Sí")</f>
         <v/>
       </c>
       <c r="E6" s="14">
-        <f>COUNTIFS('Lista 100 ml'!$B$7:$B$301,B6,'Lista 100 ml'!$H$7:$H$301,"No")</f>
+        <f>COUNTIFS('Lista 100 ml'!$B$7:$B$302,B6,'Lista 100 ml'!$H$7:$H$302,"No")</f>
         <v/>
       </c>
       <c r="F6" s="14">
-        <f>COUNTIFS('Lista 100 ml'!$B$7:$B$301,B6,'Lista 100 ml'!$I$7:$I$301,"&gt;0")</f>
+        <f>COUNTIFS('Lista 100 ml'!$B$7:$B$302,B6,'Lista 100 ml'!$I$7:$I$302,"&gt;0")</f>
         <v/>
       </c>
     </row>

</xml_diff>